<commit_message>
set soft power from wgcna signed-network heuristic and add outlier sensitivity
</commit_message>
<xml_diff>
--- a/04_Figures/F06_Prediction/c_data/F06_supplementary.xlsx
+++ b/04_Figures/F06_Prediction/c_data/F06_supplementary.xlsx
@@ -1006,7 +1006,7 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>0.73134328358209</v>
+        <v>0.791044776119403</v>
       </c>
       <c r="O3" t="s">
         <v>36</v>
@@ -1032,7 +1032,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0.243756243756244</v>
+        <v>0.23976023976024</v>
       </c>
       <c r="H4" t="n">
         <v>1000</v>
@@ -1070,16 +1070,16 @@
         <v>38</v>
       </c>
       <c r="D5" t="n">
-        <v>0.555555555555556</v>
+        <v>0.541666666666667</v>
       </c>
       <c r="E5" t="n">
-        <v>0.312077072062061</v>
+        <v>0.297083966698734</v>
       </c>
       <c r="F5" t="n">
-        <v>0.79903403904905</v>
+        <v>0.786249366634599</v>
       </c>
       <c r="G5" t="n">
-        <v>0.73134328358209</v>
+        <v>0.791044776119403</v>
       </c>
       <c r="H5" t="n">
         <v>200</v>
@@ -1100,7 +1100,7 @@
         <v>1</v>
       </c>
       <c r="N5" t="n">
-        <v>0.73134328358209</v>
+        <v>0.791044776119403</v>
       </c>
       <c r="O5" t="s">
         <v>36</v>
@@ -2485,10 +2485,10 @@
         <v>37</v>
       </c>
       <c r="C91" t="n">
-        <v>0.416666666666667</v>
+        <v>0.5</v>
       </c>
       <c r="D91" t="n">
-        <v>0.583333333333333</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="92">
@@ -2499,10 +2499,10 @@
         <v>37</v>
       </c>
       <c r="C92" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D92" t="n">
         <v>0.416666666666667</v>
-      </c>
-      <c r="D92" t="n">
-        <v>0.5</v>
       </c>
     </row>
     <row r="93">
@@ -4431,13 +4431,13 @@
         <v>87</v>
       </c>
       <c r="D2" t="n">
-        <v>0.526666666666667</v>
+        <v>0.52</v>
       </c>
       <c r="E2" t="n">
-        <v>0.506666666666667</v>
+        <v>0.513333333333333</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02</v>
+        <v>0.00666666666666659</v>
       </c>
       <c r="G2" t="n">
         <v>25</v>
@@ -4500,10 +4500,10 @@
         <v>88</v>
       </c>
       <c r="D5" t="n">
-        <v>0.593333333333333</v>
+        <v>0.58</v>
       </c>
       <c r="E5" t="n">
-        <v>0.613333333333333</v>
+        <v>0.6</v>
       </c>
       <c r="F5" t="n">
         <v>-0.0199999999999999</v>
@@ -4546,13 +4546,13 @@
         <v>87</v>
       </c>
       <c r="D7" t="n">
-        <v>0.583333333333333</v>
+        <v>0.590277777777778</v>
       </c>
       <c r="E7" t="n">
-        <v>0.555555555555556</v>
+        <v>0.569444444444444</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0277777777777777</v>
+        <v>0.0208333333333333</v>
       </c>
       <c r="G7" t="n">
         <v>24</v>
@@ -4592,13 +4592,13 @@
         <v>86</v>
       </c>
       <c r="D9" t="n">
-        <v>0.5625</v>
+        <v>0.548611111111111</v>
       </c>
       <c r="E9" t="n">
-        <v>0.5625</v>
+        <v>0.548611111111111</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.000000000000000111022302462516</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
         <v>24</v>
@@ -4615,13 +4615,13 @@
         <v>88</v>
       </c>
       <c r="D10" t="n">
-        <v>0.548611111111111</v>
+        <v>0.541666666666667</v>
       </c>
       <c r="E10" t="n">
-        <v>0.527777777777778</v>
+        <v>0.534722222222222</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0208333333333333</v>
+        <v>0.00694444444444442</v>
       </c>
       <c r="G10" t="n">
         <v>24</v>
@@ -4638,13 +4638,13 @@
         <v>106</v>
       </c>
       <c r="D11" t="n">
-        <v>0.541666666666667</v>
+        <v>0.534722222222222</v>
       </c>
       <c r="E11" t="n">
-        <v>0.527777777777778</v>
+        <v>0.534722222222222</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0138888888888888</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
         <v>24</v>
@@ -4720,22 +4720,22 @@
         <v>87</v>
       </c>
       <c r="D2" t="n">
-        <v>0.526666666666667</v>
+        <v>0.52</v>
       </c>
       <c r="E2" t="n">
         <v>0.75</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.223333333333333</v>
+        <v>-0.23</v>
       </c>
       <c r="G2" t="n">
         <v>9</v>
       </c>
       <c r="H2" t="n">
-        <v>0.349947210100793</v>
+        <v>0.353737627963812</v>
       </c>
       <c r="I2" t="n">
-        <v>0.204892966360856</v>
+        <v>0.216463414634146</v>
       </c>
       <c r="J2" t="n">
         <v>25</v>
@@ -4767,10 +4767,10 @@
         <v>25</v>
       </c>
       <c r="H3" t="n">
-        <v>0.860798372246086</v>
+        <v>0.857300124650146</v>
       </c>
       <c r="I3" t="n">
-        <v>0.729078014184397</v>
+        <v>0.725601131541726</v>
       </c>
       <c r="J3" t="n">
         <v>25</v>
@@ -4802,10 +4802,10 @@
         <v>25</v>
       </c>
       <c r="H4" t="n">
-        <v>0.605395350959709</v>
+        <v>0.610236786984455</v>
       </c>
       <c r="I4" t="n">
-        <v>0.569204152249135</v>
+        <v>0.586086956521739</v>
       </c>
       <c r="J4" t="n">
         <v>25</v>
@@ -4825,7 +4825,7 @@
         <v>88</v>
       </c>
       <c r="D5" t="n">
-        <v>0.593333333333333</v>
+        <v>0.58</v>
       </c>
       <c r="E5"/>
       <c r="F5"/>
@@ -4833,10 +4833,10 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0522434745685635</v>
+        <v>0.0558635954376046</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0425170068027211</v>
+        <v>0.0460750853242321</v>
       </c>
       <c r="J5" t="n">
         <v>25</v>
@@ -4868,10 +4868,10 @@
         <v>25</v>
       </c>
       <c r="H6" t="n">
-        <v>0.570187409680101</v>
+        <v>0.56914237602363</v>
       </c>
       <c r="I6" t="n">
-        <v>0.496923076923077</v>
+        <v>0.496111975116641</v>
       </c>
       <c r="J6" t="n">
         <v>25</v>
@@ -4891,7 +4891,7 @@
         <v>87</v>
       </c>
       <c r="D7" t="n">
-        <v>0.583333333333333</v>
+        <v>0.590277777777778</v>
       </c>
       <c r="E7"/>
       <c r="F7"/>
@@ -4899,10 +4899,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0.225356060075322</v>
+        <v>0.230293621344312</v>
       </c>
       <c r="I7" t="n">
-        <v>0.151988636363636</v>
+        <v>0.157968970380818</v>
       </c>
       <c r="J7" t="n">
         <v>12</v>
@@ -4934,10 +4934,10 @@
         <v>22</v>
       </c>
       <c r="H8" t="n">
-        <v>0.568700697055282</v>
+        <v>0.56807905929465</v>
       </c>
       <c r="I8" t="n">
-        <v>0.393557422969188</v>
+        <v>0.393006993006993</v>
       </c>
       <c r="J8" t="n">
         <v>12</v>
@@ -4957,24 +4957,24 @@
         <v>86</v>
       </c>
       <c r="D9" t="n">
-        <v>0.5625</v>
+        <v>0.548611111111111</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
       <c r="G9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H9" t="n">
-        <v>0.316696872993555</v>
+        <v>0.31143323451231</v>
       </c>
       <c r="I9" t="n">
-        <v>0.248210023866348</v>
+        <v>0.242352941176471</v>
       </c>
       <c r="J9" t="n">
         <v>12</v>
       </c>
       <c r="K9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -4988,22 +4988,22 @@
         <v>88</v>
       </c>
       <c r="D10" t="n">
-        <v>0.548611111111111</v>
+        <v>0.541666666666667</v>
       </c>
       <c r="E10" t="n">
         <v>0.612244897959184</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.0636337868480726</v>
+        <v>-0.0705782312925171</v>
       </c>
       <c r="G10" t="n">
         <v>14</v>
       </c>
       <c r="H10" t="n">
-        <v>0.440508851758479</v>
+        <v>0.437228616599428</v>
       </c>
       <c r="I10" t="n">
-        <v>0.293333333333333</v>
+        <v>0.285714285714286</v>
       </c>
       <c r="J10" t="n">
         <v>12</v>
@@ -5023,22 +5023,22 @@
         <v>106</v>
       </c>
       <c r="D11" t="n">
-        <v>0.541666666666667</v>
+        <v>0.534722222222222</v>
       </c>
       <c r="E11" t="n">
         <v>0.56198347107438</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.0203168044077133</v>
+        <v>-0.0272612488521577</v>
       </c>
       <c r="G11" t="n">
         <v>22</v>
       </c>
       <c r="H11" t="n">
-        <v>0.523230308573207</v>
+        <v>0.517141513750416</v>
       </c>
       <c r="I11" t="n">
-        <v>0.385579937304075</v>
+        <v>0.381329113924051</v>
       </c>
       <c r="J11" t="n">
         <v>12</v>
@@ -5107,16 +5107,16 @@
         <v>117</v>
       </c>
       <c r="B2" t="n">
-        <v>0.600474843402708</v>
+        <v>0.598757324712063</v>
       </c>
       <c r="C2" t="n">
-        <v>0.530880162440023</v>
+        <v>0.5293726537674</v>
       </c>
       <c r="D2" t="n">
-        <v>0.670069524365392</v>
+        <v>0.668141995656726</v>
       </c>
       <c r="E2" t="n">
-        <v>0.124378109452736</v>
+        <v>0.114427860696517</v>
       </c>
       <c r="F2" t="n">
         <v>297</v>
@@ -5128,10 +5128,10 @@
         <v>196</v>
       </c>
       <c r="I2" t="n">
-        <v>6.54295547255271</v>
+        <v>6.8475901856507</v>
       </c>
       <c r="J2" t="n">
-        <v>0.25690918004412</v>
+        <v>0.232224230554656</v>
       </c>
     </row>
   </sheetData>
@@ -5170,10 +5170,10 @@
         <v>106</v>
       </c>
       <c r="B2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -5184,10 +5184,10 @@
         <v>86</v>
       </c>
       <c r="B3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3" t="n">
         <v>3</v>
@@ -5215,7 +5215,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
         <v>2</v>
@@ -5243,7 +5243,7 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
pin the roc direction so anti-predictive models stop reading above chance
pROC was re-detecting orientation on every call, which hit the permutation
null hardest: it refits on shuffled labels, k=1 selection inverts out-of-fold,
and every anti-predictive draw got folded back over 0.5 (null mean 0.708).
Pinned, the null sits at 0.364 and module baseline lands at AUC 0.82,
perm p 0.003, q 0.018. Training arm is below chance, as it should have read
all along. uni_auc and the perm_p_* pair stay on auto on purpose, since an
eigengene's sign is arbitrary and they fold obs and null together.
</commit_message>
<xml_diff>
--- a/04_Figures/F06_Prediction/c_data/F06_supplementary.xlsx
+++ b/04_Figures/F06_Prediction/c_data/F06_supplementary.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
   <si>
     <t xml:space="preserve">F06 Prediction — supplementary tables</t>
   </si>
@@ -139,6 +139,9 @@
   </si>
   <si>
     <t xml:space="preserve">module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*</t>
   </si>
   <si>
     <t xml:space="preserve">hallmark</t>
@@ -938,7 +941,7 @@
         <v>0.99233259131192</v>
       </c>
       <c r="G2" t="n">
-        <v>0.17910447761194</v>
+        <v>0.0845771144278607</v>
       </c>
       <c r="H2" t="n">
         <v>200</v>
@@ -959,7 +962,7 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>0.641791044776119</v>
+        <v>0.169154228855721</v>
       </c>
       <c r="O2" t="s">
         <v>36</v>
@@ -976,16 +979,16 @@
         <v>38</v>
       </c>
       <c r="D3" t="n">
-        <v>0.611111111111111</v>
+        <v>0.388888888888889</v>
       </c>
       <c r="E3" t="n">
-        <v>0.372664872878278</v>
+        <v>0.150442650656055</v>
       </c>
       <c r="F3" t="n">
-        <v>0.849557349343944</v>
+        <v>0.627335127121722</v>
       </c>
       <c r="G3" t="n">
-        <v>0.686567164179104</v>
+        <v>0.6318407960199</v>
       </c>
       <c r="H3" t="n">
         <v>200</v>
@@ -1006,7 +1009,7 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>0.791044776119403</v>
+        <v>0.75820895522388</v>
       </c>
       <c r="O3" t="s">
         <v>36</v>
@@ -1032,7 +1035,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0.23976023976024</v>
+        <v>0.00299700299700299</v>
       </c>
       <c r="H4" t="n">
         <v>1000</v>
@@ -1053,10 +1056,10 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>0.641791044776119</v>
+        <v>0.017982017982018</v>
       </c>
       <c r="O4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -1070,16 +1073,16 @@
         <v>38</v>
       </c>
       <c r="D5" t="n">
-        <v>0.541666666666667</v>
+        <v>0.458333333333333</v>
       </c>
       <c r="E5" t="n">
-        <v>0.297083966698734</v>
+        <v>0.213750633365401</v>
       </c>
       <c r="F5" t="n">
-        <v>0.786249366634599</v>
+        <v>0.702916033301266</v>
       </c>
       <c r="G5" t="n">
-        <v>0.791044776119403</v>
+        <v>0.54228855721393</v>
       </c>
       <c r="H5" t="n">
         <v>200</v>
@@ -1100,7 +1103,7 @@
         <v>1</v>
       </c>
       <c r="N5" t="n">
-        <v>0.791044776119403</v>
+        <v>0.75820895522388</v>
       </c>
       <c r="O5" t="s">
         <v>36</v>
@@ -1108,7 +1111,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B6" t="s">
         <v>34</v>
@@ -1126,7 +1129,7 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>0.393034825870647</v>
+        <v>0.0845771144278607</v>
       </c>
       <c r="H6" t="n">
         <v>200</v>
@@ -1147,7 +1150,7 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>0.641791044776119</v>
+        <v>0.169154228855721</v>
       </c>
       <c r="O6" t="s">
         <v>36</v>
@@ -1155,7 +1158,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
         <v>37</v>
@@ -1164,16 +1167,16 @@
         <v>38</v>
       </c>
       <c r="D7" t="n">
-        <v>0.645833333333333</v>
+        <v>0.354166666666667</v>
       </c>
       <c r="E7" t="n">
-        <v>0.413758265507818</v>
+        <v>0.122091598841151</v>
       </c>
       <c r="F7" t="n">
-        <v>0.877908401158849</v>
+        <v>0.586241734492182</v>
       </c>
       <c r="G7" t="n">
-        <v>0.427860696517413</v>
+        <v>0.776119402985075</v>
       </c>
       <c r="H7" t="n">
         <v>200</v>
@@ -1194,7 +1197,7 @@
         <v>1</v>
       </c>
       <c r="N7" t="n">
-        <v>0.641791044776119</v>
+        <v>0.776119402985075</v>
       </c>
       <c r="O7" t="s">
         <v>36</v>
@@ -1225,10 +1228,10 @@
         <v>19</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2">
@@ -1617,10 +1620,10 @@
         <v>37</v>
       </c>
       <c r="C29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
         <v>0.916666666666667</v>
-      </c>
-      <c r="D29" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -1631,10 +1634,10 @@
         <v>37</v>
       </c>
       <c r="C30" t="n">
-        <v>0.916666666666667</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>0.916666666666667</v>
+        <v>0.833333333333333</v>
       </c>
     </row>
     <row r="31">
@@ -1645,10 +1648,10 @@
         <v>37</v>
       </c>
       <c r="C31" t="n">
-        <v>0.833333333333333</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>0.916666666666667</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="32">
@@ -1659,10 +1662,10 @@
         <v>37</v>
       </c>
       <c r="C32" t="n">
+        <v>0.916666666666667</v>
+      </c>
+      <c r="D32" t="n">
         <v>0.75</v>
-      </c>
-      <c r="D32" t="n">
-        <v>0.916666666666667</v>
       </c>
     </row>
     <row r="33">
@@ -1673,10 +1676,10 @@
         <v>37</v>
       </c>
       <c r="C33" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="D33" t="n">
-        <v>0.916666666666667</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="34">
@@ -1687,10 +1690,10 @@
         <v>37</v>
       </c>
       <c r="C34" t="n">
-        <v>0.583333333333333</v>
+        <v>0.75</v>
       </c>
       <c r="D34" t="n">
-        <v>0.916666666666667</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="35">
@@ -1701,10 +1704,10 @@
         <v>37</v>
       </c>
       <c r="C35" t="n">
-        <v>0.583333333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="D35" t="n">
-        <v>0.833333333333333</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="36">
@@ -1715,10 +1718,10 @@
         <v>37</v>
       </c>
       <c r="C36" t="n">
-        <v>0.583333333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="D36" t="n">
-        <v>0.75</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="37">
@@ -1729,10 +1732,10 @@
         <v>37</v>
       </c>
       <c r="C37" t="n">
+        <v>0.666666666666667</v>
+      </c>
+      <c r="D37" t="n">
         <v>0.583333333333333</v>
-      </c>
-      <c r="D37" t="n">
-        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="38">
@@ -1743,10 +1746,10 @@
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>0.583333333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="D38" t="n">
-        <v>0.583333333333333</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="39">
@@ -1757,10 +1760,10 @@
         <v>37</v>
       </c>
       <c r="C39" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="D39" t="n">
         <v>0.5</v>
-      </c>
-      <c r="D39" t="n">
-        <v>0.583333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -1771,10 +1774,10 @@
         <v>37</v>
       </c>
       <c r="C40" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="D40" t="n">
         <v>0.416666666666667</v>
-      </c>
-      <c r="D40" t="n">
-        <v>0.583333333333333</v>
       </c>
     </row>
     <row r="41">
@@ -1785,10 +1788,10 @@
         <v>37</v>
       </c>
       <c r="C41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D41" t="n">
         <v>0.416666666666667</v>
-      </c>
-      <c r="D41" t="n">
-        <v>0.5</v>
       </c>
     </row>
     <row r="42">
@@ -1799,10 +1802,10 @@
         <v>37</v>
       </c>
       <c r="C42" t="n">
-        <v>0.333333333333333</v>
+        <v>0.416666666666667</v>
       </c>
       <c r="D42" t="n">
-        <v>0.5</v>
+        <v>0.416666666666667</v>
       </c>
     </row>
     <row r="43">
@@ -1813,10 +1816,10 @@
         <v>37</v>
       </c>
       <c r="C43" t="n">
+        <v>0.416666666666667</v>
+      </c>
+      <c r="D43" t="n">
         <v>0.333333333333333</v>
-      </c>
-      <c r="D43" t="n">
-        <v>0.416666666666667</v>
       </c>
     </row>
     <row r="44">
@@ -1827,10 +1830,10 @@
         <v>37</v>
       </c>
       <c r="C44" t="n">
-        <v>0.333333333333333</v>
+        <v>0.416666666666667</v>
       </c>
       <c r="D44" t="n">
-        <v>0.333333333333333</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="45">
@@ -1841,10 +1844,10 @@
         <v>37</v>
       </c>
       <c r="C45" t="n">
-        <v>0.333333333333333</v>
+        <v>0.416666666666667</v>
       </c>
       <c r="D45" t="n">
-        <v>0.25</v>
+        <v>0.166666666666667</v>
       </c>
     </row>
     <row r="46">
@@ -1855,10 +1858,10 @@
         <v>37</v>
       </c>
       <c r="C46" t="n">
-        <v>0.25</v>
+        <v>0.416666666666667</v>
       </c>
       <c r="D46" t="n">
-        <v>0.25</v>
+        <v>0.0833333333333333</v>
       </c>
     </row>
     <row r="47">
@@ -1869,10 +1872,10 @@
         <v>37</v>
       </c>
       <c r="C47" t="n">
-        <v>0.166666666666667</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="D47" t="n">
-        <v>0.25</v>
+        <v>0.0833333333333333</v>
       </c>
     </row>
     <row r="48">
@@ -1883,10 +1886,10 @@
         <v>37</v>
       </c>
       <c r="C48" t="n">
-        <v>0.0833333333333334</v>
+        <v>0.25</v>
       </c>
       <c r="D48" t="n">
-        <v>0.25</v>
+        <v>0.0833333333333333</v>
       </c>
     </row>
     <row r="49">
@@ -1897,10 +1900,10 @@
         <v>37</v>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="D49" t="n">
-        <v>0.25</v>
+        <v>0.0833333333333333</v>
       </c>
     </row>
     <row r="50">
@@ -1911,10 +1914,10 @@
         <v>37</v>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>0.0833333333333334</v>
       </c>
       <c r="D50" t="n">
-        <v>0.166666666666667</v>
+        <v>0.0833333333333333</v>
       </c>
     </row>
     <row r="51">
@@ -1925,10 +1928,10 @@
         <v>37</v>
       </c>
       <c r="C51" t="n">
+        <v>0.0833333333333334</v>
+      </c>
+      <c r="D51" t="n">
         <v>0</v>
-      </c>
-      <c r="D51" t="n">
-        <v>0.0833333333333333</v>
       </c>
     </row>
     <row r="52">
@@ -2359,10 +2362,10 @@
         <v>37</v>
       </c>
       <c r="C82" t="n">
+        <v>0.916666666666667</v>
+      </c>
+      <c r="D82" t="n">
         <v>0.833333333333333</v>
-      </c>
-      <c r="D82" t="n">
-        <v>0.916666666666667</v>
       </c>
     </row>
     <row r="83">
@@ -2373,10 +2376,10 @@
         <v>37</v>
       </c>
       <c r="C83" t="n">
-        <v>0.75</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="D83" t="n">
-        <v>0.916666666666667</v>
+        <v>0.833333333333333</v>
       </c>
     </row>
     <row r="84">
@@ -2387,10 +2390,10 @@
         <v>37</v>
       </c>
       <c r="C84" t="n">
+        <v>0.833333333333333</v>
+      </c>
+      <c r="D84" t="n">
         <v>0.75</v>
-      </c>
-      <c r="D84" t="n">
-        <v>0.833333333333333</v>
       </c>
     </row>
     <row r="85">
@@ -2429,10 +2432,10 @@
         <v>37</v>
       </c>
       <c r="C87" t="n">
-        <v>0.583333333333333</v>
+        <v>0.666666666666667</v>
       </c>
       <c r="D87" t="n">
-        <v>0.75</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="88">
@@ -2443,10 +2446,10 @@
         <v>37</v>
       </c>
       <c r="C88" t="n">
-        <v>0.5</v>
+        <v>0.583333333333333</v>
       </c>
       <c r="D88" t="n">
-        <v>0.75</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="89">
@@ -2457,10 +2460,10 @@
         <v>37</v>
       </c>
       <c r="C89" t="n">
-        <v>0.5</v>
+        <v>0.583333333333333</v>
       </c>
       <c r="D89" t="n">
-        <v>0.666666666666667</v>
+        <v>0.583333333333333</v>
       </c>
     </row>
     <row r="90">
@@ -2513,10 +2516,10 @@
         <v>37</v>
       </c>
       <c r="C93" t="n">
-        <v>0.416666666666667</v>
+        <v>0.5</v>
       </c>
       <c r="D93" t="n">
-        <v>0.416666666666667</v>
+        <v>0.333333333333333</v>
       </c>
     </row>
     <row r="94">
@@ -2527,10 +2530,10 @@
         <v>37</v>
       </c>
       <c r="C94" t="n">
-        <v>0.416666666666667</v>
+        <v>0.5</v>
       </c>
       <c r="D94" t="n">
-        <v>0.333333333333333</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="95">
@@ -2541,10 +2544,10 @@
         <v>37</v>
       </c>
       <c r="C95" t="n">
-        <v>0.333333333333333</v>
+        <v>0.416666666666667</v>
       </c>
       <c r="D95" t="n">
-        <v>0.333333333333333</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="96">
@@ -2583,10 +2586,10 @@
         <v>37</v>
       </c>
       <c r="C98" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D98" t="n">
         <v>0.166666666666667</v>
-      </c>
-      <c r="D98" t="n">
-        <v>0.25</v>
       </c>
     </row>
     <row r="99">
@@ -2597,10 +2600,10 @@
         <v>37</v>
       </c>
       <c r="C99" t="n">
-        <v>0.166666666666667</v>
+        <v>0.25</v>
       </c>
       <c r="D99" t="n">
-        <v>0.166666666666667</v>
+        <v>0.0833333333333333</v>
       </c>
     </row>
     <row r="100">
@@ -2611,10 +2614,10 @@
         <v>37</v>
       </c>
       <c r="C100" t="n">
-        <v>0.0833333333333334</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="D100" t="n">
-        <v>0.166666666666667</v>
+        <v>0.0833333333333333</v>
       </c>
     </row>
     <row r="101">
@@ -2661,7 +2664,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B104" t="s">
         <v>34</v>
@@ -2675,7 +2678,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B105" t="s">
         <v>34</v>
@@ -2689,7 +2692,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B106" t="s">
         <v>34</v>
@@ -2703,7 +2706,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B107" t="s">
         <v>34</v>
@@ -2717,7 +2720,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B108" t="s">
         <v>34</v>
@@ -2731,7 +2734,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B109" t="s">
         <v>34</v>
@@ -2745,7 +2748,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B110" t="s">
         <v>34</v>
@@ -2759,7 +2762,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B111" t="s">
         <v>34</v>
@@ -2773,7 +2776,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B112" t="s">
         <v>34</v>
@@ -2787,7 +2790,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B113" t="s">
         <v>34</v>
@@ -2801,7 +2804,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B114" t="s">
         <v>34</v>
@@ -2815,7 +2818,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B115" t="s">
         <v>34</v>
@@ -2829,7 +2832,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B116" t="s">
         <v>34</v>
@@ -2843,7 +2846,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B117" t="s">
         <v>34</v>
@@ -2857,7 +2860,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B118" t="s">
         <v>34</v>
@@ -2871,7 +2874,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B119" t="s">
         <v>34</v>
@@ -2885,7 +2888,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B120" t="s">
         <v>34</v>
@@ -2899,7 +2902,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B121" t="s">
         <v>34</v>
@@ -2913,7 +2916,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B122" t="s">
         <v>34</v>
@@ -2927,7 +2930,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B123" t="s">
         <v>34</v>
@@ -2941,7 +2944,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B124" t="s">
         <v>34</v>
@@ -2955,7 +2958,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B125" t="s">
         <v>34</v>
@@ -2969,7 +2972,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B126" t="s">
         <v>34</v>
@@ -2983,7 +2986,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B127" t="s">
         <v>34</v>
@@ -2997,7 +3000,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B128" t="s">
         <v>34</v>
@@ -3011,7 +3014,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B129" t="s">
         <v>34</v>
@@ -3025,7 +3028,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B130" t="s">
         <v>37</v>
@@ -3039,63 +3042,63 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B131" t="s">
         <v>37</v>
       </c>
       <c r="C131" t="n">
+        <v>1</v>
+      </c>
+      <c r="D131" t="n">
         <v>0.916666666666667</v>
-      </c>
-      <c r="D131" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B132" t="s">
         <v>37</v>
       </c>
       <c r="C132" t="n">
+        <v>1</v>
+      </c>
+      <c r="D132" t="n">
         <v>0.833333333333333</v>
-      </c>
-      <c r="D132" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B133" t="s">
         <v>37</v>
       </c>
       <c r="C133" t="n">
-        <v>0.833333333333333</v>
+        <v>1</v>
       </c>
       <c r="D133" t="n">
-        <v>0.916666666666667</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B134" t="s">
         <v>37</v>
       </c>
       <c r="C134" t="n">
-        <v>0.833333333333333</v>
+        <v>0.916666666666667</v>
       </c>
       <c r="D134" t="n">
-        <v>0.833333333333333</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B135" t="s">
         <v>37</v>
@@ -3109,189 +3112,189 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B136" t="s">
         <v>37</v>
       </c>
       <c r="C136" t="n">
-        <v>0.75</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="D136" t="n">
-        <v>0.75</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B137" t="s">
         <v>37</v>
       </c>
       <c r="C137" t="n">
-        <v>0.666666666666667</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="D137" t="n">
-        <v>0.75</v>
+        <v>0.583333333333333</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B138" t="s">
         <v>37</v>
       </c>
       <c r="C138" t="n">
-        <v>0.583333333333333</v>
+        <v>0.833333333333333</v>
       </c>
       <c r="D138" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B139" t="s">
         <v>37</v>
       </c>
       <c r="C139" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D139" t="n">
         <v>0.5</v>
-      </c>
-      <c r="D139" t="n">
-        <v>0.75</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B140" t="s">
         <v>37</v>
       </c>
       <c r="C140" t="n">
+        <v>0.666666666666667</v>
+      </c>
+      <c r="D140" t="n">
         <v>0.5</v>
-      </c>
-      <c r="D140" t="n">
-        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B141" t="s">
         <v>37</v>
       </c>
       <c r="C141" t="n">
+        <v>0.666666666666667</v>
+      </c>
+      <c r="D141" t="n">
         <v>0.416666666666667</v>
-      </c>
-      <c r="D141" t="n">
-        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B142" t="s">
         <v>37</v>
       </c>
       <c r="C142" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="D142" t="n">
         <v>0.416666666666667</v>
-      </c>
-      <c r="D142" t="n">
-        <v>0.583333333333333</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B143" t="s">
         <v>37</v>
       </c>
       <c r="C143" t="n">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="D143" t="n">
         <v>0.333333333333333</v>
-      </c>
-      <c r="D143" t="n">
-        <v>0.583333333333333</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B144" t="s">
         <v>37</v>
       </c>
       <c r="C144" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D144" t="n">
         <v>0.333333333333333</v>
-      </c>
-      <c r="D144" t="n">
-        <v>0.5</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B145" t="s">
         <v>37</v>
       </c>
       <c r="C145" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D145" t="n">
         <v>0.25</v>
-      </c>
-      <c r="D145" t="n">
-        <v>0.5</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B146" t="s">
         <v>37</v>
       </c>
       <c r="C146" t="n">
-        <v>0.166666666666667</v>
+        <v>0.416666666666667</v>
       </c>
       <c r="D146" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B147" t="s">
         <v>37</v>
       </c>
       <c r="C147" t="n">
-        <v>0.166666666666667</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="D147" t="n">
-        <v>0.416666666666667</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B148" t="s">
         <v>37</v>
       </c>
       <c r="C148" t="n">
-        <v>0.166666666666667</v>
+        <v>0.25</v>
       </c>
       <c r="D148" t="n">
-        <v>0.333333333333333</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B149" t="s">
         <v>37</v>
@@ -3305,63 +3308,63 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B150" t="s">
         <v>37</v>
       </c>
       <c r="C150" t="n">
-        <v>0.0833333333333334</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="D150" t="n">
-        <v>0.25</v>
+        <v>0.166666666666667</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B151" t="s">
         <v>37</v>
       </c>
       <c r="C151" t="n">
-        <v>0</v>
+        <v>0.166666666666667</v>
       </c>
       <c r="D151" t="n">
-        <v>0.25</v>
+        <v>0.0833333333333333</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B152" t="s">
         <v>37</v>
       </c>
       <c r="C152" t="n">
+        <v>0.166666666666667</v>
+      </c>
+      <c r="D152" t="n">
         <v>0</v>
-      </c>
-      <c r="D152" t="n">
-        <v>0.166666666666667</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B153" t="s">
         <v>37</v>
       </c>
       <c r="C153" t="n">
+        <v>0.0833333333333334</v>
+      </c>
+      <c r="D153" t="n">
         <v>0</v>
-      </c>
-      <c r="D153" t="n">
-        <v>0.0833333333333333</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B154" t="s">
         <v>37</v>
@@ -3399,13 +3402,13 @@
         <v>19</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2">
@@ -3416,7 +3419,7 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D2" t="n">
         <v>22</v>
@@ -3433,7 +3436,7 @@
         <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D3" t="n">
         <v>19</v>
@@ -3450,7 +3453,7 @@
         <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D4" t="n">
         <v>11</v>
@@ -3467,7 +3470,7 @@
         <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D5" t="n">
         <v>10</v>
@@ -3484,7 +3487,7 @@
         <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D6" t="n">
         <v>5</v>
@@ -3501,7 +3504,7 @@
         <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D7" t="n">
         <v>4</v>
@@ -3518,7 +3521,7 @@
         <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D8" t="n">
         <v>4</v>
@@ -3535,7 +3538,7 @@
         <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D9" t="n">
         <v>3</v>
@@ -3552,7 +3555,7 @@
         <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D10" t="n">
         <v>3</v>
@@ -3569,7 +3572,7 @@
         <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D11" t="n">
         <v>3</v>
@@ -3586,7 +3589,7 @@
         <v>34</v>
       </c>
       <c r="C12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D12" t="n">
         <v>3</v>
@@ -3603,7 +3606,7 @@
         <v>34</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D13" t="n">
         <v>3</v>
@@ -3620,7 +3623,7 @@
         <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D14" t="n">
         <v>2</v>
@@ -3637,7 +3640,7 @@
         <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D15" t="n">
         <v>2</v>
@@ -3654,7 +3657,7 @@
         <v>34</v>
       </c>
       <c r="C16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
@@ -3671,7 +3674,7 @@
         <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D17" t="n">
         <v>1</v>
@@ -3688,7 +3691,7 @@
         <v>34</v>
       </c>
       <c r="C18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
@@ -3705,7 +3708,7 @@
         <v>34</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
@@ -3722,7 +3725,7 @@
         <v>34</v>
       </c>
       <c r="C20" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D20" t="n">
         <v>1</v>
@@ -3739,7 +3742,7 @@
         <v>34</v>
       </c>
       <c r="C21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D21" t="n">
         <v>1</v>
@@ -3756,7 +3759,7 @@
         <v>37</v>
       </c>
       <c r="C22" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D22" t="n">
         <v>12</v>
@@ -3773,7 +3776,7 @@
         <v>37</v>
       </c>
       <c r="C23" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D23" t="n">
         <v>4</v>
@@ -3790,7 +3793,7 @@
         <v>37</v>
       </c>
       <c r="C24" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D24" t="n">
         <v>3</v>
@@ -3807,7 +3810,7 @@
         <v>37</v>
       </c>
       <c r="C25" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D25" t="n">
         <v>3</v>
@@ -3824,7 +3827,7 @@
         <v>37</v>
       </c>
       <c r="C26" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D26" t="n">
         <v>2</v>
@@ -3841,7 +3844,7 @@
         <v>37</v>
       </c>
       <c r="C27" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D27" t="n">
         <v>2</v>
@@ -3858,7 +3861,7 @@
         <v>37</v>
       </c>
       <c r="C28" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D28" t="n">
         <v>1</v>
@@ -3875,7 +3878,7 @@
         <v>37</v>
       </c>
       <c r="C29" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D29" t="n">
         <v>1</v>
@@ -3892,7 +3895,7 @@
         <v>37</v>
       </c>
       <c r="C30" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D30" t="n">
         <v>1</v>
@@ -3909,7 +3912,7 @@
         <v>37</v>
       </c>
       <c r="C31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D31" t="n">
         <v>1</v>
@@ -3926,7 +3929,7 @@
         <v>37</v>
       </c>
       <c r="C32" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D32" t="n">
         <v>1</v>
@@ -3943,7 +3946,7 @@
         <v>37</v>
       </c>
       <c r="C33" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D33" t="n">
         <v>1</v>
@@ -3960,7 +3963,7 @@
         <v>37</v>
       </c>
       <c r="C34" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D34" t="n">
         <v>1</v>
@@ -3977,7 +3980,7 @@
         <v>37</v>
       </c>
       <c r="C35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D35" t="n">
         <v>1</v>
@@ -3994,7 +3997,7 @@
         <v>37</v>
       </c>
       <c r="C36" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D36" t="n">
         <v>1</v>
@@ -4011,7 +4014,7 @@
         <v>37</v>
       </c>
       <c r="C37" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D37" t="n">
         <v>1</v>
@@ -4028,7 +4031,7 @@
         <v>37</v>
       </c>
       <c r="C38" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D38" t="n">
         <v>1</v>
@@ -4045,7 +4048,7 @@
         <v>37</v>
       </c>
       <c r="C39" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D39" t="n">
         <v>1</v>
@@ -4062,7 +4065,7 @@
         <v>37</v>
       </c>
       <c r="C40" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D40" t="n">
         <v>1</v>
@@ -4079,7 +4082,7 @@
         <v>34</v>
       </c>
       <c r="C41" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D41" t="n">
         <v>25</v>
@@ -4096,7 +4099,7 @@
         <v>34</v>
       </c>
       <c r="C42" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D42" t="n">
         <v>1</v>
@@ -4113,7 +4116,7 @@
         <v>37</v>
       </c>
       <c r="C43" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D43" t="n">
         <v>10</v>
@@ -4130,7 +4133,7 @@
         <v>37</v>
       </c>
       <c r="C44" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D44" t="n">
         <v>4</v>
@@ -4141,13 +4144,13 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B45" t="s">
         <v>34</v>
       </c>
       <c r="C45" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D45" t="n">
         <v>25</v>
@@ -4158,13 +4161,13 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B46" t="s">
         <v>34</v>
       </c>
       <c r="C46" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D46" t="n">
         <v>3</v>
@@ -4175,13 +4178,13 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B47" t="s">
         <v>34</v>
       </c>
       <c r="C47" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D47" t="n">
         <v>1</v>
@@ -4192,13 +4195,13 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B48" t="s">
         <v>34</v>
       </c>
       <c r="C48" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D48" t="n">
         <v>1</v>
@@ -4209,13 +4212,13 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B49" t="s">
         <v>34</v>
       </c>
       <c r="C49" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D49" t="n">
         <v>1</v>
@@ -4226,13 +4229,13 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B50" t="s">
         <v>34</v>
       </c>
       <c r="C50" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D50" t="n">
         <v>1</v>
@@ -4243,13 +4246,13 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B51" t="s">
         <v>34</v>
       </c>
       <c r="C51" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D51" t="n">
         <v>1</v>
@@ -4260,13 +4263,13 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B52" t="s">
         <v>34</v>
       </c>
       <c r="C52" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D52" t="n">
         <v>1</v>
@@ -4277,13 +4280,13 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B53" t="s">
         <v>34</v>
       </c>
       <c r="C53" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D53" t="n">
         <v>1</v>
@@ -4294,13 +4297,13 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B54" t="s">
         <v>34</v>
       </c>
       <c r="C54" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D54" t="n">
         <v>1</v>
@@ -4311,13 +4314,13 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B55" t="s">
         <v>37</v>
       </c>
       <c r="C55" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D55" t="n">
         <v>7</v>
@@ -4328,13 +4331,13 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B56" t="s">
         <v>37</v>
       </c>
       <c r="C56" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D56" t="n">
         <v>4</v>
@@ -4345,13 +4348,13 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B57" t="s">
         <v>37</v>
       </c>
       <c r="C57" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D57" t="n">
         <v>1</v>
@@ -4362,13 +4365,13 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B58" t="s">
         <v>37</v>
       </c>
       <c r="C58" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D58" t="n">
         <v>1</v>
@@ -4399,7 +4402,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>19</v>
@@ -4408,13 +4411,13 @@
         <v>39</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>27</v>
@@ -4422,13 +4425,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D2" t="n">
         <v>0.52</v>
@@ -4445,13 +4448,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D3" t="n">
         <v>0.96</v>
@@ -4468,13 +4471,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B4" t="s">
         <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D4" t="n">
         <v>0.853333333333333</v>
@@ -4491,13 +4494,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B5" t="s">
         <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D5" t="n">
         <v>0.58</v>
@@ -4514,13 +4517,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B6" t="s">
         <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D6" t="n">
         <v>0.813333333333333</v>
@@ -4537,13 +4540,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B7" t="s">
         <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D7" t="n">
         <v>0.590277777777778</v>
@@ -4560,13 +4563,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B8" t="s">
         <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D8" t="n">
         <v>0.576388888888889</v>
@@ -4583,13 +4586,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B9" t="s">
         <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D9" t="n">
         <v>0.548611111111111</v>
@@ -4606,13 +4609,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B10" t="s">
         <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D10" t="n">
         <v>0.541666666666667</v>
@@ -4629,13 +4632,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B11" t="s">
         <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D11" t="n">
         <v>0.534722222222222</v>
@@ -4676,7 +4679,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>19</v>
@@ -4685,39 +4688,39 @@
         <v>39</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>27</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D2" t="n">
         <v>0.52</v>
@@ -4746,13 +4749,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D3" t="n">
         <v>0.96</v>
@@ -4781,13 +4784,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B4" t="s">
         <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D4" t="n">
         <v>0.853333333333333</v>
@@ -4816,13 +4819,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B5" t="s">
         <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D5" t="n">
         <v>0.58</v>
@@ -4847,13 +4850,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B6" t="s">
         <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D6" t="n">
         <v>0.813333333333333</v>
@@ -4882,13 +4885,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B7" t="s">
         <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D7" t="n">
         <v>0.590277777777778</v>
@@ -4913,13 +4916,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B8" t="s">
         <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D8" t="n">
         <v>0.576388888888889</v>
@@ -4948,13 +4951,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B9" t="s">
         <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D9" t="n">
         <v>0.548611111111111</v>
@@ -4979,13 +4982,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B10" t="s">
         <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D10" t="n">
         <v>0.541666666666667</v>
@@ -5014,13 +5017,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B11" t="s">
         <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D11" t="n">
         <v>0.534722222222222</v>
@@ -5072,7 +5075,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>21</v>
@@ -5090,21 +5093,21 @@
         <v>27</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B2" t="n">
         <v>0.598757324712063</v>
@@ -5116,7 +5119,7 @@
         <v>0.668141995656726</v>
       </c>
       <c r="E2" t="n">
-        <v>0.114427860696517</v>
+        <v>0.0149253731343283</v>
       </c>
       <c r="F2" t="n">
         <v>297</v>
@@ -5153,21 +5156,21 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B2" t="n">
         <v>19</v>
@@ -5181,7 +5184,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B3" t="n">
         <v>14</v>
@@ -5195,7 +5198,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B4" t="n">
         <v>1</v>
@@ -5209,7 +5212,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B5" t="n">
         <v>4</v>
@@ -5223,7 +5226,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B6" t="n">
         <v>63</v>
@@ -5237,7 +5240,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
read the wgcna soft power off disk instead of guessing 12 when it is 14
</commit_message>
<xml_diff>
--- a/04_Figures/F06_Prediction/c_data/F06_supplementary.xlsx
+++ b/04_Figures/F06_Prediction/c_data/F06_supplementary.xlsx
@@ -4735,10 +4735,10 @@
         <v>9</v>
       </c>
       <c r="H2" t="n">
-        <v>0.353737627963812</v>
+        <v>0.359166900463107</v>
       </c>
       <c r="I2" t="n">
-        <v>0.216463414634146</v>
+        <v>0.218446601941748</v>
       </c>
       <c r="J2" t="n">
         <v>25</v>
@@ -4770,10 +4770,10 @@
         <v>25</v>
       </c>
       <c r="H3" t="n">
-        <v>0.857300124650146</v>
+        <v>0.852175494545965</v>
       </c>
       <c r="I3" t="n">
-        <v>0.725601131541726</v>
+        <v>0.705965909090909</v>
       </c>
       <c r="J3" t="n">
         <v>25</v>
@@ -4796,19 +4796,19 @@
         <v>0.853333333333333</v>
       </c>
       <c r="E4" t="n">
-        <v>0.853333333333333</v>
+        <v>0.86</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>-0.00666666666666659</v>
       </c>
       <c r="G4" t="n">
         <v>25</v>
       </c>
       <c r="H4" t="n">
-        <v>0.610236786984455</v>
+        <v>0.602798665043135</v>
       </c>
       <c r="I4" t="n">
-        <v>0.586086956521739</v>
+        <v>0.568259385665529</v>
       </c>
       <c r="J4" t="n">
         <v>25</v>
@@ -4836,10 +4836,10 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0558635954376046</v>
+        <v>0.0567826109842718</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0460750853242321</v>
+        <v>0.0498281786941581</v>
       </c>
       <c r="J5" t="n">
         <v>25</v>
@@ -4862,19 +4862,19 @@
         <v>0.813333333333333</v>
       </c>
       <c r="E6" t="n">
-        <v>0.793333333333333</v>
+        <v>0.8</v>
       </c>
       <c r="F6" t="n">
-        <v>0.02</v>
+        <v>0.0133333333333333</v>
       </c>
       <c r="G6" t="n">
         <v>25</v>
       </c>
       <c r="H6" t="n">
-        <v>0.56914237602363</v>
+        <v>0.566799416293588</v>
       </c>
       <c r="I6" t="n">
-        <v>0.496111975116641</v>
+        <v>0.483024691358025</v>
       </c>
       <c r="J6" t="n">
         <v>25</v>
@@ -4899,19 +4899,19 @@
       <c r="E7"/>
       <c r="F7"/>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H7" t="n">
-        <v>0.230293621344312</v>
+        <v>0.273534005524309</v>
       </c>
       <c r="I7" t="n">
-        <v>0.157968970380818</v>
+        <v>0.162659123055163</v>
       </c>
       <c r="J7" t="n">
         <v>12</v>
       </c>
       <c r="K7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -4928,25 +4928,25 @@
         <v>0.576388888888889</v>
       </c>
       <c r="E8" t="n">
-        <v>0.644628099173554</v>
+        <v>0.576388888888889</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.0682392102846648</v>
+        <v>0.000000000000000111022302462516</v>
       </c>
       <c r="G8" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H8" t="n">
-        <v>0.56807905929465</v>
+        <v>0.567852397440105</v>
       </c>
       <c r="I8" t="n">
-        <v>0.393006993006993</v>
+        <v>0.419667590027701</v>
       </c>
       <c r="J8" t="n">
         <v>12</v>
       </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -4962,22 +4962,26 @@
       <c r="D9" t="n">
         <v>0.548611111111111</v>
       </c>
-      <c r="E9"/>
-      <c r="F9"/>
+      <c r="E9" t="n">
+        <v>0.888888888888889</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-0.340277777777778</v>
+      </c>
       <c r="G9" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H9" t="n">
-        <v>0.31143323451231</v>
+        <v>0.347761799740051</v>
       </c>
       <c r="I9" t="n">
-        <v>0.242352941176471</v>
+        <v>0.259958071278826</v>
       </c>
       <c r="J9" t="n">
         <v>12</v>
       </c>
       <c r="K9" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -4994,19 +4998,19 @@
         <v>0.541666666666667</v>
       </c>
       <c r="E10" t="n">
-        <v>0.612244897959184</v>
+        <v>0.551020408163265</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.0705782312925171</v>
+        <v>-0.00935374149659873</v>
       </c>
       <c r="G10" t="n">
         <v>14</v>
       </c>
       <c r="H10" t="n">
-        <v>0.437228616599428</v>
+        <v>0.410096334666936</v>
       </c>
       <c r="I10" t="n">
-        <v>0.285714285714286</v>
+        <v>0.305555555555556</v>
       </c>
       <c r="J10" t="n">
         <v>12</v>
@@ -5029,19 +5033,19 @@
         <v>0.534722222222222</v>
       </c>
       <c r="E11" t="n">
-        <v>0.56198347107438</v>
+        <v>0.537190082644628</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.0272612488521577</v>
+        <v>-0.00246786042240576</v>
       </c>
       <c r="G11" t="n">
         <v>22</v>
       </c>
       <c r="H11" t="n">
-        <v>0.517141513750416</v>
+        <v>0.510540315479178</v>
       </c>
       <c r="I11" t="n">
-        <v>0.381329113924051</v>
+        <v>0.351910828025478</v>
       </c>
       <c r="J11" t="n">
         <v>12</v>

</xml_diff>